<commit_message>
Update raw data inventory
NCDOT PBIN and RoadNC data update
</commit_message>
<xml_diff>
--- a/raw_source_inventory.xlsx
+++ b/raw_source_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jliu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://centralina-my.sharepoint.com/personal/jliu_centralina_org/Documents/Desktop/mh_explorer/git_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA357D76-74AB-4C8A-858B-68E9C7BEB4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{FA357D76-74AB-4C8A-858B-68E9C7BEB4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9785565D-76B7-4AB7-952A-353183066198}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="1480" windowWidth="14400" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Sources" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="369">
   <si>
     <t>Raw Data Source Inventory</t>
   </si>
@@ -517,9 +517,6 @@
     <t>pbin</t>
   </si>
   <si>
-    <t>NCDOT- Pedestrian and Bike Infrastructure Network, July 2024</t>
-  </si>
-  <si>
     <t>pedestrian, bike infrastructure</t>
   </si>
   <si>
@@ -1121,6 +1118,15 @@
   </si>
   <si>
     <t>Service-area polygons for GoGastonia based on website description, used to map the geographic coverage of on-demand microtransit service.</t>
+  </si>
+  <si>
+    <t>the raw dataset updates quarterly. The 2026 version is from March 2026.</t>
+  </si>
+  <si>
+    <t>NCDOT- Pedestrian and Bike Infrastructure Network, July 2026</t>
+  </si>
+  <si>
+    <t>the most recent dataset is from July 2026.</t>
   </si>
 </sst>
 </file>
@@ -1387,11 +1393,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R60"/>
-  <sheetFormatPr defaultColWidth="32.25" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="32.25" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="17.4140625" customWidth="1"/>
-    <col min="2" max="2" width="20.1640625" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.375" customWidth="1"/>
+    <col min="2" max="2" width="20.125" customWidth="1"/>
+    <col min="3" max="3" width="21.375" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="14" width="9.25" customWidth="1"/>
   </cols>
@@ -1465,7 +1471,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="32" customHeight="1">
+    <row r="4" spans="1:18" ht="32.1" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -1476,7 +1482,7 @@
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>19</v>
@@ -1508,7 +1514,7 @@
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:18" ht="32" customHeight="1">
+    <row r="5" spans="1:18" ht="32.1" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -1519,7 +1525,7 @@
         <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>19</v>
@@ -1551,7 +1557,7 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:18" ht="32" customHeight="1">
+    <row r="6" spans="1:18" ht="32.1" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -1562,7 +1568,7 @@
         <v>30</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>19</v>
@@ -1594,7 +1600,7 @@
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="1:18" ht="32" customHeight="1">
+    <row r="7" spans="1:18" ht="32.1" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
@@ -1605,7 +1611,7 @@
         <v>30</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>19</v>
@@ -1637,7 +1643,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:18" ht="32" customHeight="1">
+    <row r="8" spans="1:18" ht="32.1" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
@@ -1648,7 +1654,7 @@
         <v>37</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>38</v>
@@ -1680,7 +1686,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:18" ht="32" customHeight="1">
+    <row r="9" spans="1:18" ht="32.1" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>42</v>
       </c>
@@ -1691,7 +1697,7 @@
         <v>44</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>45</v>
@@ -1727,7 +1733,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="32" customHeight="1">
+    <row r="10" spans="1:18" ht="32.1" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>42</v>
       </c>
@@ -1738,7 +1744,7 @@
         <v>53</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
@@ -1774,7 +1780,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="32" customHeight="1">
+    <row r="11" spans="1:18" ht="32.1" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>60</v>
       </c>
@@ -1785,7 +1791,7 @@
         <v>62</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>63</v>
@@ -1819,7 +1825,7 @@
       </c>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:18" ht="32" customHeight="1">
+    <row r="12" spans="1:18" ht="32.1" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
@@ -1830,7 +1836,7 @@
         <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>63</v>
@@ -1864,7 +1870,7 @@
       </c>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:18" ht="32" customHeight="1">
+    <row r="13" spans="1:18" ht="32.1" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1875,7 +1881,7 @@
         <v>71</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>63</v>
@@ -1909,7 +1915,7 @@
       </c>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:18" ht="32" customHeight="1">
+    <row r="14" spans="1:18" ht="32.1" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>60</v>
       </c>
@@ -1920,7 +1926,7 @@
         <v>71</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>63</v>
@@ -1954,7 +1960,7 @@
       </c>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:18" ht="32" customHeight="1">
+    <row r="15" spans="1:18" ht="32.1" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>60</v>
       </c>
@@ -1965,7 +1971,7 @@
         <v>71</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>63</v>
@@ -1999,7 +2005,7 @@
       </c>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:18" ht="32" customHeight="1">
+    <row r="16" spans="1:18" ht="32.1" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>60</v>
       </c>
@@ -2010,7 +2016,7 @@
         <v>71</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>63</v>
@@ -2044,7 +2050,7 @@
       </c>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="1:15" ht="32" customHeight="1">
+    <row r="17" spans="1:15" ht="32.1" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -2055,7 +2061,7 @@
         <v>92</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>63</v>
@@ -2089,7 +2095,7 @@
       </c>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="1:15" ht="32" customHeight="1">
+    <row r="18" spans="1:15" ht="32.1" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>60</v>
       </c>
@@ -2100,7 +2106,7 @@
         <v>71</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>63</v>
@@ -2134,7 +2140,7 @@
       </c>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="1:15" ht="32" customHeight="1">
+    <row r="19" spans="1:15" ht="32.1" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
@@ -2145,7 +2151,7 @@
         <v>92</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>63</v>
@@ -2179,7 +2185,7 @@
       </c>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="1:15" ht="32" customHeight="1">
+    <row r="20" spans="1:15" ht="32.1" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>60</v>
       </c>
@@ -2190,7 +2196,7 @@
         <v>53</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -2226,7 +2232,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="32" customHeight="1">
+    <row r="21" spans="1:15" ht="32.1" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>107</v>
       </c>
@@ -2237,7 +2243,7 @@
         <v>109</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>110</v>
@@ -2273,7 +2279,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="32" customHeight="1">
+    <row r="22" spans="1:15" ht="32.1" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -2284,7 +2290,7 @@
         <v>109</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>110</v>
@@ -2320,7 +2326,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="32" customHeight="1">
+    <row r="23" spans="1:15" ht="32.1" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>115</v>
       </c>
@@ -2331,7 +2337,7 @@
         <v>119</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>110</v>
@@ -2365,7 +2371,7 @@
       </c>
       <c r="O23" s="2"/>
     </row>
-    <row r="24" spans="1:15" ht="32" customHeight="1">
+    <row r="24" spans="1:15" ht="32.1" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>115</v>
       </c>
@@ -2376,7 +2382,7 @@
         <v>125</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>63</v>
@@ -2410,7 +2416,7 @@
       </c>
       <c r="O24" s="2"/>
     </row>
-    <row r="25" spans="1:15" ht="32" customHeight="1">
+    <row r="25" spans="1:15" ht="32.1" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>115</v>
       </c>
@@ -2421,7 +2427,7 @@
         <v>125</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>63</v>
@@ -2455,7 +2461,7 @@
       </c>
       <c r="O25" s="2"/>
     </row>
-    <row r="26" spans="1:15" ht="32" customHeight="1">
+    <row r="26" spans="1:15" ht="32.1" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>115</v>
       </c>
@@ -2466,7 +2472,7 @@
         <v>135</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>63</v>
@@ -2500,7 +2506,7 @@
       </c>
       <c r="O26" s="2"/>
     </row>
-    <row r="27" spans="1:15" ht="32" customHeight="1">
+    <row r="27" spans="1:15" ht="32.1" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>115</v>
       </c>
@@ -2511,7 +2517,7 @@
         <v>135</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>63</v>
@@ -2545,7 +2551,7 @@
       </c>
       <c r="O27" s="2"/>
     </row>
-    <row r="28" spans="1:15" ht="32" customHeight="1">
+    <row r="28" spans="1:15" ht="32.1" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>115</v>
       </c>
@@ -2556,7 +2562,7 @@
         <v>135</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>63</v>
@@ -2590,7 +2596,7 @@
       </c>
       <c r="O28" s="2"/>
     </row>
-    <row r="29" spans="1:15" ht="32" customHeight="1">
+    <row r="29" spans="1:15" ht="32.1" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>115</v>
       </c>
@@ -2601,7 +2607,7 @@
         <v>148</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>63</v>
@@ -2635,7 +2641,7 @@
       </c>
       <c r="O29" s="2"/>
     </row>
-    <row r="30" spans="1:15" ht="32" customHeight="1">
+    <row r="30" spans="1:15" ht="32.1" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>115</v>
       </c>
@@ -2646,7 +2652,7 @@
         <v>154</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>63</v>
@@ -2680,7 +2686,7 @@
       </c>
       <c r="O30" s="2"/>
     </row>
-    <row r="31" spans="1:15" ht="32" customHeight="1">
+    <row r="31" spans="1:15" ht="32.1" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>159</v>
       </c>
@@ -2691,7 +2697,7 @@
         <v>148</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>110</v>
@@ -2721,9 +2727,11 @@
         <v>162</v>
       </c>
       <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
-    </row>
-    <row r="32" spans="1:15" ht="32" customHeight="1">
+      <c r="O31" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="32.1" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>163</v>
       </c>
@@ -2731,10 +2739,10 @@
         <v>164</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>165</v>
+        <v>367</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2743,50 +2751,52 @@
         <v>149</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>55</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>24</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>26</v>
       </c>
       <c r="M32" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="N32" s="2"/>
+      <c r="O32" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A33" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-    </row>
-    <row r="33" spans="1:15" ht="32" customHeight="1">
-      <c r="A33" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="D33" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F33" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>65</v>
@@ -2795,43 +2805,43 @@
         <v>56</v>
       </c>
       <c r="J33" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="K33" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="K33" s="2" t="s">
+      <c r="L33" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M33" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M33" s="2" t="s">
+      <c r="N33" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="N33" s="2" t="s">
+      <c r="O33" s="2"/>
+    </row>
+    <row r="34" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="O33" s="2"/>
-    </row>
-    <row r="34" spans="1:15" ht="32" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="D34" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F34" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>65</v>
@@ -2840,43 +2850,43 @@
         <v>66</v>
       </c>
       <c r="J34" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M34" s="2" t="s">
+      <c r="N34" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="N34" s="2" t="s">
+      <c r="O34" s="2"/>
+    </row>
+    <row r="35" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="O34" s="2"/>
-    </row>
-    <row r="35" spans="1:15" ht="32" customHeight="1">
-      <c r="A35" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>184</v>
-      </c>
       <c r="D35" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>65</v>
@@ -2885,7 +2895,7 @@
         <v>56</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>25</v>
@@ -2894,34 +2904,34 @@
         <v>26</v>
       </c>
       <c r="M35" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="N35" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="N35" s="2" t="s">
+      <c r="O35" s="2"/>
+    </row>
+    <row r="36" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="O35" s="2"/>
-    </row>
-    <row r="36" spans="1:15" ht="32" customHeight="1">
-      <c r="A36" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>189</v>
-      </c>
       <c r="C36" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>65</v>
@@ -2930,7 +2940,7 @@
         <v>66</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>25</v>
@@ -2939,34 +2949,34 @@
         <v>26</v>
       </c>
       <c r="M36" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="N36" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="N36" s="2" t="s">
+      <c r="O36" s="2"/>
+    </row>
+    <row r="37" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="O36" s="2"/>
-    </row>
-    <row r="37" spans="1:15" ht="32" customHeight="1">
-      <c r="A37" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>193</v>
-      </c>
       <c r="C37" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>65</v>
@@ -2975,7 +2985,7 @@
         <v>56</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>25</v>
@@ -2984,34 +2994,34 @@
         <v>26</v>
       </c>
       <c r="M37" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="N37" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="N37" s="2" t="s">
+      <c r="O37" s="2"/>
+    </row>
+    <row r="38" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="O37" s="2"/>
-    </row>
-    <row r="38" spans="1:15" ht="32" customHeight="1">
-      <c r="A38" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="C38" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>65</v>
@@ -3020,7 +3030,7 @@
         <v>66</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>25</v>
@@ -3029,34 +3039,34 @@
         <v>26</v>
       </c>
       <c r="M38" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="N38" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="N38" s="2" t="s">
+      <c r="O38" s="2"/>
+    </row>
+    <row r="39" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="O38" s="2"/>
-    </row>
-    <row r="39" spans="1:15" ht="32" customHeight="1">
-      <c r="A39" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="C39" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>65</v>
@@ -3065,7 +3075,7 @@
         <v>56</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>25</v>
@@ -3074,34 +3084,34 @@
         <v>26</v>
       </c>
       <c r="M39" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="N39" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="N39" s="2" t="s">
+      <c r="O39" s="2"/>
+    </row>
+    <row r="40" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="O39" s="2"/>
-    </row>
-    <row r="40" spans="1:15" ht="32" customHeight="1">
-      <c r="A40" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>205</v>
-      </c>
       <c r="C40" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>65</v>
@@ -3110,7 +3120,7 @@
         <v>66</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>25</v>
@@ -3119,34 +3129,34 @@
         <v>26</v>
       </c>
       <c r="M40" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="N40" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="N40" s="2" t="s">
+      <c r="O40" s="2"/>
+    </row>
+    <row r="41" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="O40" s="2"/>
-    </row>
-    <row r="41" spans="1:15" ht="32" customHeight="1">
-      <c r="A41" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>209</v>
-      </c>
       <c r="C41" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>65</v>
@@ -3155,7 +3165,7 @@
         <v>56</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>25</v>
@@ -3164,34 +3174,34 @@
         <v>26</v>
       </c>
       <c r="M41" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="N41" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="N41" s="2" t="s">
+      <c r="O41" s="2"/>
+    </row>
+    <row r="42" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="O41" s="2"/>
-    </row>
-    <row r="42" spans="1:15" ht="32" customHeight="1">
-      <c r="A42" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>214</v>
-      </c>
       <c r="C42" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>65</v>
@@ -3200,7 +3210,7 @@
         <v>66</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K42" s="2" t="s">
         <v>25</v>
@@ -3209,34 +3219,34 @@
         <v>26</v>
       </c>
       <c r="M42" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="N42" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="N42" s="2" t="s">
+      <c r="O42" s="2"/>
+    </row>
+    <row r="43" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="O42" s="2"/>
-    </row>
-    <row r="43" spans="1:15" ht="32" customHeight="1">
-      <c r="A43" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>218</v>
-      </c>
       <c r="C43" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>65</v>
@@ -3245,7 +3255,7 @@
         <v>56</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>25</v>
@@ -3254,34 +3264,34 @@
         <v>26</v>
       </c>
       <c r="M43" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="N43" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="N43" s="2" t="s">
+      <c r="O43" s="2"/>
+    </row>
+    <row r="44" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="O43" s="2"/>
-    </row>
-    <row r="44" spans="1:15" ht="32" customHeight="1">
-      <c r="A44" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>222</v>
-      </c>
       <c r="C44" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>65</v>
@@ -3290,7 +3300,7 @@
         <v>66</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>25</v>
@@ -3299,34 +3309,34 @@
         <v>26</v>
       </c>
       <c r="M44" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="N44" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="N44" s="2" t="s">
+      <c r="O44" s="2"/>
+    </row>
+    <row r="45" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="O44" s="2"/>
-    </row>
-    <row r="45" spans="1:15" ht="32" customHeight="1">
-      <c r="A45" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>226</v>
-      </c>
       <c r="C45" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>65</v>
@@ -3335,7 +3345,7 @@
         <v>56</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>25</v>
@@ -3344,34 +3354,34 @@
         <v>26</v>
       </c>
       <c r="M45" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="N45" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="N45" s="2" t="s">
+      <c r="O45" s="2"/>
+    </row>
+    <row r="46" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="O45" s="2"/>
-    </row>
-    <row r="46" spans="1:15" ht="32" customHeight="1">
-      <c r="A46" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="C46" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>65</v>
@@ -3380,7 +3390,7 @@
         <v>66</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>25</v>
@@ -3389,34 +3399,34 @@
         <v>26</v>
       </c>
       <c r="M46" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="N46" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="N46" s="2" t="s">
+      <c r="O46" s="2"/>
+    </row>
+    <row r="47" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="O46" s="2"/>
-    </row>
-    <row r="47" spans="1:15" ht="32" customHeight="1">
-      <c r="A47" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>235</v>
-      </c>
       <c r="D47" s="4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F47" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>65</v>
@@ -3425,7 +3435,7 @@
         <v>56</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>25</v>
@@ -3434,34 +3444,34 @@
         <v>26</v>
       </c>
       <c r="M47" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="N47" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="N47" s="2" t="s">
+      <c r="O47" s="2"/>
+    </row>
+    <row r="48" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="O47" s="2"/>
-    </row>
-    <row r="48" spans="1:15" ht="32" customHeight="1">
-      <c r="A48" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>241</v>
-      </c>
       <c r="C48" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F48" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>65</v>
@@ -3470,7 +3480,7 @@
         <v>66</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>25</v>
@@ -3479,43 +3489,43 @@
         <v>26</v>
       </c>
       <c r="M48" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="N48" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="N48" s="2" t="s">
+      <c r="O48" s="2"/>
+    </row>
+    <row r="49" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="O48" s="2"/>
-    </row>
-    <row r="49" spans="1:15" ht="32" customHeight="1">
-      <c r="A49" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B49" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="D49" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="E49" s="2" t="s">
+      <c r="F49" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="G49" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H49" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="G49" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="H49" s="2" t="s">
+      <c r="I49" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="J49" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="I49" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="J49" s="2" t="s">
-        <v>250</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>48</v>
@@ -3524,43 +3534,43 @@
         <v>26</v>
       </c>
       <c r="M49" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="O49" s="2"/>
+    </row>
+    <row r="50" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="N49" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="O49" s="2"/>
-    </row>
-    <row r="50" spans="1:15" ht="32" customHeight="1">
-      <c r="A50" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="C50" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F50" s="2" t="s">
+      <c r="G50" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="J50" s="2" t="s">
         <v>253</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>48</v>
@@ -3569,43 +3579,43 @@
         <v>26</v>
       </c>
       <c r="M50" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="O50" s="2"/>
+    </row>
+    <row r="51" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="N50" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="O50" s="2"/>
-    </row>
-    <row r="51" spans="1:15" ht="32" customHeight="1">
-      <c r="A51" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B51" s="2" t="s">
+      <c r="C51" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F51" s="2" t="s">
+      <c r="G51" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="H51" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="J51" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="J51" s="2" t="s">
-        <v>259</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>48</v>
@@ -3614,43 +3624,43 @@
         <v>26</v>
       </c>
       <c r="M51" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="O51" s="2"/>
+    </row>
+    <row r="52" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="N51" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="O51" s="2"/>
-    </row>
-    <row r="52" spans="1:15" ht="32" customHeight="1">
-      <c r="A52" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B52" s="2" t="s">
+      <c r="C52" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F52" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F52" s="2" t="s">
+      <c r="G52" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="J52" s="2" t="s">
         <v>262</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="I52" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="J52" s="2" t="s">
-        <v>263</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>48</v>
@@ -3659,43 +3669,43 @@
         <v>26</v>
       </c>
       <c r="M52" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O52" s="2"/>
+    </row>
+    <row r="53" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="N52" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="O52" s="2"/>
-    </row>
-    <row r="53" spans="1:15" ht="32" customHeight="1">
-      <c r="A53" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B53" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="D53" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="D53" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F53" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="H53" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="H53" s="2" t="s">
+      <c r="I53" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="J53" s="2" t="s">
         <v>269</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>270</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>48</v>
@@ -3704,41 +3714,41 @@
         <v>26</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="1:15" ht="32" customHeight="1">
+    <row r="54" spans="1:15" ht="32.1" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="D54" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D54" s="4" t="s">
-        <v>351</v>
-      </c>
-      <c r="E54" s="2" t="s">
+      <c r="F54" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="G54" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="J54" s="2" t="s">
         <v>275</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="I54" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="J54" s="2" t="s">
-        <v>276</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>48</v>
@@ -3747,41 +3757,41 @@
         <v>26</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="1:15" ht="32" customHeight="1">
+    <row r="55" spans="1:15" ht="32.1" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="C55" s="2" t="s">
-        <v>279</v>
-      </c>
       <c r="D55" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>55</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>48</v>
@@ -3790,32 +3800,32 @@
         <v>26</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
     </row>
-    <row r="56" spans="1:15" ht="32" customHeight="1">
+    <row r="56" spans="1:15" ht="32.1" customHeight="1">
       <c r="A56" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>283</v>
-      </c>
       <c r="C56" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F56" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>285</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>65</v>
@@ -3824,43 +3834,43 @@
         <v>23</v>
       </c>
       <c r="J56" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M56" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="K56" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M56" s="2" t="s">
+      <c r="N56" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="N56" s="2" t="s">
+      <c r="O56" s="2"/>
+    </row>
+    <row r="57" spans="1:15" ht="32.1" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="O56" s="2"/>
-    </row>
-    <row r="57" spans="1:15" ht="32" customHeight="1">
-      <c r="A57" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="B57" s="2" t="s">
+      <c r="C57" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>290</v>
-      </c>
       <c r="D57" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>110</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>112</v>
@@ -3869,7 +3879,7 @@
         <v>23</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>25</v>
@@ -3878,32 +3888,32 @@
         <v>26</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="1:15" ht="32" customHeight="1">
+    <row r="58" spans="1:15" ht="32.1" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B58" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>295</v>
-      </c>
       <c r="D58" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>110</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>112</v>
@@ -3912,7 +3922,7 @@
         <v>23</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>25</v>
@@ -3921,32 +3931,32 @@
         <v>26</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="1:15" ht="32" customHeight="1">
+    <row r="59" spans="1:15" ht="32.1" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>300</v>
-      </c>
       <c r="D59" s="4" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>110</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>112</v>
@@ -3955,7 +3965,7 @@
         <v>23</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>25</v>
@@ -3964,32 +3974,32 @@
         <v>26</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
     </row>
-    <row r="60" spans="1:15" ht="32" customHeight="1">
+    <row r="60" spans="1:15" ht="32.1" customHeight="1">
       <c r="A60" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>305</v>
-      </c>
       <c r="C60" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>65</v>
@@ -3998,19 +4008,19 @@
         <v>66</v>
       </c>
       <c r="J60" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M60" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="K60" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M60" s="2" t="s">
+      <c r="N60" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="N60" s="2" t="s">
-        <v>309</v>
       </c>
       <c r="O60" s="2"/>
     </row>

</xml_diff>

<commit_message>
update log and inventory
</commit_message>
<xml_diff>
--- a/raw_source_inventory.xlsx
+++ b/raw_source_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://centralina-my.sharepoint.com/personal/jliu_centralina_org/Documents/Desktop/mh_explorer/git_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{FA357D76-74AB-4C8A-858B-68E9C7BEB4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9785565D-76B7-4AB7-952A-353183066198}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{FA357D76-74AB-4C8A-858B-68E9C7BEB4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91B93D2C-8A80-4002-A4D0-23E702BB2449}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Sources" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="368">
   <si>
     <t>Raw Data Source Inventory</t>
   </si>
@@ -532,9 +532,6 @@
     <t>routes_bus_cats</t>
   </si>
   <si>
-    <t>CATS, 2026 April</t>
-  </si>
-  <si>
     <t>CATS</t>
   </si>
   <si>
@@ -556,9 +553,6 @@
     <t>stops_bus_cats</t>
   </si>
   <si>
-    <t>CATS, 2026 May</t>
-  </si>
-  <si>
     <t>cats_sc</t>
   </si>
   <si>
@@ -1127,13 +1121,16 @@
   </si>
   <si>
     <t>the most recent dataset is from July 2026.</t>
+  </si>
+  <si>
+    <t>CATS, 2026 August</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1154,6 +1151,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1183,10 +1186,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1203,8 +1207,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1220,8 +1228,19 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RawSourcesTable" displayName="RawSourcesTable" ref="A3:O60">
+  <autoFilter ref="A3:O60" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="monthly"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Source Group"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Raw Item ID"/>
@@ -1471,7 +1490,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="32.1" customHeight="1">
+    <row r="4" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -1482,7 +1501,7 @@
         <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>19</v>
@@ -1514,7 +1533,7 @@
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:18" ht="32.1" customHeight="1">
+    <row r="5" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -1525,7 +1544,7 @@
         <v>30</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>19</v>
@@ -1557,7 +1576,7 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:18" ht="32.1" customHeight="1">
+    <row r="6" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -1568,7 +1587,7 @@
         <v>30</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>19</v>
@@ -1600,7 +1619,7 @@
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="1:18" ht="32.1" customHeight="1">
+    <row r="7" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
@@ -1611,7 +1630,7 @@
         <v>30</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>19</v>
@@ -1643,7 +1662,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:18" ht="32.1" customHeight="1">
+    <row r="8" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
@@ -1654,7 +1673,7 @@
         <v>37</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>38</v>
@@ -1686,7 +1705,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:18" ht="32.1" customHeight="1">
+    <row r="9" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>42</v>
       </c>
@@ -1697,7 +1716,7 @@
         <v>44</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>45</v>
@@ -1733,7 +1752,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="32.1" customHeight="1">
+    <row r="10" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>42</v>
       </c>
@@ -1744,7 +1763,7 @@
         <v>53</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>54</v>
@@ -1780,7 +1799,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="32.1" customHeight="1">
+    <row r="11" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>60</v>
       </c>
@@ -1791,7 +1810,7 @@
         <v>62</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>63</v>
@@ -1825,7 +1844,7 @@
       </c>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:18" ht="32.1" customHeight="1">
+    <row r="12" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
@@ -1836,7 +1855,7 @@
         <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>63</v>
@@ -1870,7 +1889,7 @@
       </c>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:18" ht="32.1" customHeight="1">
+    <row r="13" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1881,7 +1900,7 @@
         <v>71</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>63</v>
@@ -1915,7 +1934,7 @@
       </c>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:18" ht="32.1" customHeight="1">
+    <row r="14" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>60</v>
       </c>
@@ -1926,7 +1945,7 @@
         <v>71</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>63</v>
@@ -1960,7 +1979,7 @@
       </c>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:18" ht="32.1" customHeight="1">
+    <row r="15" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>60</v>
       </c>
@@ -1971,7 +1990,7 @@
         <v>71</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>63</v>
@@ -2005,7 +2024,7 @@
       </c>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:18" ht="32.1" customHeight="1">
+    <row r="16" spans="1:18" ht="32.1" hidden="1" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>60</v>
       </c>
@@ -2016,7 +2035,7 @@
         <v>71</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>63</v>
@@ -2050,7 +2069,7 @@
       </c>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="1:15" ht="32.1" customHeight="1">
+    <row r="17" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -2061,7 +2080,7 @@
         <v>92</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>63</v>
@@ -2095,7 +2114,7 @@
       </c>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="1:15" ht="32.1" customHeight="1">
+    <row r="18" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>60</v>
       </c>
@@ -2106,7 +2125,7 @@
         <v>71</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>63</v>
@@ -2140,7 +2159,7 @@
       </c>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="1:15" ht="32.1" customHeight="1">
+    <row r="19" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
@@ -2151,7 +2170,7 @@
         <v>92</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>63</v>
@@ -2185,7 +2204,7 @@
       </c>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="1:15" ht="32.1" customHeight="1">
+    <row r="20" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>60</v>
       </c>
@@ -2196,7 +2215,7 @@
         <v>53</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>54</v>
@@ -2232,7 +2251,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="32.1" customHeight="1">
+    <row r="21" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>107</v>
       </c>
@@ -2243,7 +2262,7 @@
         <v>109</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>110</v>
@@ -2279,7 +2298,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="32.1" customHeight="1">
+    <row r="22" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -2290,7 +2309,7 @@
         <v>109</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>110</v>
@@ -2326,7 +2345,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="32.1" customHeight="1">
+    <row r="23" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>115</v>
       </c>
@@ -2337,7 +2356,7 @@
         <v>119</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>110</v>
@@ -2371,7 +2390,7 @@
       </c>
       <c r="O23" s="2"/>
     </row>
-    <row r="24" spans="1:15" ht="32.1" customHeight="1">
+    <row r="24" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>115</v>
       </c>
@@ -2382,7 +2401,7 @@
         <v>125</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>63</v>
@@ -2416,7 +2435,7 @@
       </c>
       <c r="O24" s="2"/>
     </row>
-    <row r="25" spans="1:15" ht="32.1" customHeight="1">
+    <row r="25" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>115</v>
       </c>
@@ -2427,7 +2446,7 @@
         <v>125</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>63</v>
@@ -2461,7 +2480,7 @@
       </c>
       <c r="O25" s="2"/>
     </row>
-    <row r="26" spans="1:15" ht="32.1" customHeight="1">
+    <row r="26" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>115</v>
       </c>
@@ -2472,7 +2491,7 @@
         <v>135</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>63</v>
@@ -2506,7 +2525,7 @@
       </c>
       <c r="O26" s="2"/>
     </row>
-    <row r="27" spans="1:15" ht="32.1" customHeight="1">
+    <row r="27" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>115</v>
       </c>
@@ -2517,7 +2536,7 @@
         <v>135</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>63</v>
@@ -2551,7 +2570,7 @@
       </c>
       <c r="O27" s="2"/>
     </row>
-    <row r="28" spans="1:15" ht="32.1" customHeight="1">
+    <row r="28" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>115</v>
       </c>
@@ -2562,7 +2581,7 @@
         <v>135</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>63</v>
@@ -2596,7 +2615,7 @@
       </c>
       <c r="O28" s="2"/>
     </row>
-    <row r="29" spans="1:15" ht="32.1" customHeight="1">
+    <row r="29" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>115</v>
       </c>
@@ -2607,7 +2626,7 @@
         <v>148</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>63</v>
@@ -2641,7 +2660,7 @@
       </c>
       <c r="O29" s="2"/>
     </row>
-    <row r="30" spans="1:15" ht="32.1" customHeight="1">
+    <row r="30" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>115</v>
       </c>
@@ -2652,7 +2671,7 @@
         <v>154</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>63</v>
@@ -2686,7 +2705,7 @@
       </c>
       <c r="O30" s="2"/>
     </row>
-    <row r="31" spans="1:15" ht="32.1" customHeight="1">
+    <row r="31" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>159</v>
       </c>
@@ -2697,7 +2716,7 @@
         <v>148</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>110</v>
@@ -2728,10 +2747,10 @@
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" ht="32.1" customHeight="1">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>163</v>
       </c>
@@ -2739,10 +2758,10 @@
         <v>164</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>54</v>
@@ -2773,7 +2792,7 @@
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="33" spans="1:15" ht="32.1" customHeight="1">
@@ -2784,19 +2803,19 @@
         <v>169</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>170</v>
+        <v>367</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F33" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>172</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>65</v>
@@ -2805,19 +2824,19 @@
         <v>56</v>
       </c>
       <c r="J33" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="K33" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="K33" s="2" t="s">
+      <c r="L33" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M33" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M33" s="2" t="s">
+      <c r="N33" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="O33" s="2"/>
     </row>
@@ -2826,22 +2845,22 @@
         <v>168</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>178</v>
+        <v>367</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F34" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>172</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>65</v>
@@ -2850,43 +2869,43 @@
         <v>66</v>
       </c>
       <c r="J34" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="N34" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>181</v>
-      </c>
       <c r="O34" s="2"/>
     </row>
-    <row r="35" spans="1:15" ht="32.1" customHeight="1">
+    <row r="35" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>65</v>
@@ -2895,7 +2914,7 @@
         <v>56</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>25</v>
@@ -2904,34 +2923,34 @@
         <v>26</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="O35" s="2"/>
     </row>
-    <row r="36" spans="1:15" ht="32.1" customHeight="1">
+    <row r="36" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>65</v>
@@ -2940,7 +2959,7 @@
         <v>66</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>25</v>
@@ -2949,34 +2968,34 @@
         <v>26</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="O36" s="2"/>
     </row>
-    <row r="37" spans="1:15" ht="32.1" customHeight="1">
+    <row r="37" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>65</v>
@@ -2985,7 +3004,7 @@
         <v>56</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>25</v>
@@ -2994,34 +3013,34 @@
         <v>26</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="O37" s="2"/>
     </row>
-    <row r="38" spans="1:15" ht="32.1" customHeight="1">
+    <row r="38" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>65</v>
@@ -3030,7 +3049,7 @@
         <v>66</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>25</v>
@@ -3039,34 +3058,34 @@
         <v>26</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="O38" s="2"/>
     </row>
-    <row r="39" spans="1:15" ht="32.1" customHeight="1">
+    <row r="39" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>65</v>
@@ -3075,7 +3094,7 @@
         <v>56</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>25</v>
@@ -3084,34 +3103,34 @@
         <v>26</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="O39" s="2"/>
     </row>
-    <row r="40" spans="1:15" ht="32.1" customHeight="1">
+    <row r="40" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>65</v>
@@ -3120,7 +3139,7 @@
         <v>66</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>25</v>
@@ -3129,34 +3148,34 @@
         <v>26</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="O40" s="2"/>
     </row>
-    <row r="41" spans="1:15" ht="32.1" customHeight="1">
+    <row r="41" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>65</v>
@@ -3165,7 +3184,7 @@
         <v>56</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>25</v>
@@ -3174,34 +3193,34 @@
         <v>26</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="O41" s="2"/>
     </row>
-    <row r="42" spans="1:15" ht="32.1" customHeight="1">
+    <row r="42" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>65</v>
@@ -3210,7 +3229,7 @@
         <v>66</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K42" s="2" t="s">
         <v>25</v>
@@ -3219,34 +3238,34 @@
         <v>26</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="O42" s="2"/>
     </row>
-    <row r="43" spans="1:15" ht="32.1" customHeight="1">
+    <row r="43" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>65</v>
@@ -3255,7 +3274,7 @@
         <v>56</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>25</v>
@@ -3264,34 +3283,34 @@
         <v>26</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="O43" s="2"/>
     </row>
-    <row r="44" spans="1:15" ht="32.1" customHeight="1">
+    <row r="44" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>65</v>
@@ -3300,7 +3319,7 @@
         <v>66</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>25</v>
@@ -3309,34 +3328,34 @@
         <v>26</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="O44" s="2"/>
     </row>
-    <row r="45" spans="1:15" ht="32.1" customHeight="1">
+    <row r="45" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>65</v>
@@ -3345,7 +3364,7 @@
         <v>56</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>25</v>
@@ -3354,34 +3373,34 @@
         <v>26</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="O45" s="2"/>
     </row>
-    <row r="46" spans="1:15" ht="32.1" customHeight="1">
+    <row r="46" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>65</v>
@@ -3390,7 +3409,7 @@
         <v>66</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>25</v>
@@ -3399,34 +3418,34 @@
         <v>26</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="O46" s="2"/>
     </row>
-    <row r="47" spans="1:15" ht="32.1" customHeight="1">
+    <row r="47" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>65</v>
@@ -3435,7 +3454,7 @@
         <v>56</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>25</v>
@@ -3444,34 +3463,34 @@
         <v>26</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="O47" s="2"/>
     </row>
-    <row r="48" spans="1:15" ht="32.1" customHeight="1">
+    <row r="48" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>65</v>
@@ -3480,7 +3499,7 @@
         <v>66</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>25</v>
@@ -3489,43 +3508,43 @@
         <v>26</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="O48" s="2"/>
     </row>
-    <row r="49" spans="1:15" ht="32.1" customHeight="1">
+    <row r="49" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="F49" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="E49" s="2" t="s">
+      <c r="G49" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H49" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>166</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>48</v>
@@ -3534,43 +3553,43 @@
         <v>26</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="1:15" ht="32.1" customHeight="1">
+    <row r="50" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H50" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>166</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>48</v>
@@ -3579,43 +3598,43 @@
         <v>26</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="O50" s="2"/>
     </row>
-    <row r="51" spans="1:15" ht="32.1" customHeight="1">
+    <row r="51" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G51" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="E51" s="2" t="s">
+      <c r="H51" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>166</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>48</v>
@@ -3624,43 +3643,43 @@
         <v>26</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="O51" s="2"/>
     </row>
-    <row r="52" spans="1:15" ht="32.1" customHeight="1">
+    <row r="52" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E52" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H52" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>166</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>48</v>
@@ -3669,43 +3688,43 @@
         <v>26</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="O52" s="2"/>
     </row>
-    <row r="53" spans="1:15" ht="32.1" customHeight="1">
+    <row r="53" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="F53" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="G53" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D53" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F53" s="2" t="s">
+      <c r="H53" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>268</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>166</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>48</v>
@@ -3714,41 +3733,41 @@
         <v>26</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="1:15" ht="32.1" customHeight="1">
+    <row r="54" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="F54" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D54" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>274</v>
-      </c>
       <c r="G54" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>166</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>48</v>
@@ -3757,32 +3776,32 @@
         <v>26</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="1:15" ht="32.1" customHeight="1">
+    <row r="55" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A55" s="2" t="s">
         <v>168</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>54</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>55</v>
@@ -3791,7 +3810,7 @@
         <v>166</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>48</v>
@@ -3800,32 +3819,32 @@
         <v>26</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
     </row>
     <row r="56" spans="1:15" ht="32.1" customHeight="1">
       <c r="A56" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>170</v>
+        <v>367</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>65</v>
@@ -3834,43 +3853,43 @@
         <v>23</v>
       </c>
       <c r="J56" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M56" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="N56" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="K56" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M56" s="2" t="s">
+      <c r="O56" s="2"/>
+    </row>
+    <row r="57" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="N56" s="2" t="s">
+      <c r="C57" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="O56" s="2"/>
-    </row>
-    <row r="57" spans="1:15" ht="32.1" customHeight="1">
-      <c r="A57" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>289</v>
-      </c>
       <c r="D57" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>110</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>112</v>
@@ -3879,7 +3898,7 @@
         <v>23</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>25</v>
@@ -3888,32 +3907,32 @@
         <v>26</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="1:15" ht="32.1" customHeight="1">
+    <row r="58" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>110</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>112</v>
@@ -3922,7 +3941,7 @@
         <v>23</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>25</v>
@@ -3931,32 +3950,32 @@
         <v>26</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="1:15" ht="32.1" customHeight="1">
+    <row r="59" spans="1:15" ht="32.1" hidden="1" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>110</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>112</v>
@@ -3965,7 +3984,7 @@
         <v>23</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>25</v>
@@ -3974,32 +3993,32 @@
         <v>26</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
     </row>
     <row r="60" spans="1:15" ht="32.1" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>170</v>
+        <v>367</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>65</v>
@@ -4008,19 +4027,19 @@
         <v>66</v>
       </c>
       <c r="J60" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="N60" s="6" t="s">
         <v>306</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="N60" s="2" t="s">
-        <v>308</v>
       </c>
       <c r="O60" s="2"/>
     </row>
@@ -4028,9 +4047,14 @@
   <mergeCells count="1">
     <mergeCell ref="A1:R1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="M33" r:id="rId1" xr:uid="{8BB7A647-2DDA-4ED6-AE50-03F3477D183F}"/>
+    <hyperlink ref="M56" r:id="rId2" xr:uid="{96EB0AB1-62A8-42AB-890F-8B0360FA9177}"/>
+    <hyperlink ref="N60" r:id="rId3" xr:uid="{24594A1D-A61B-4026-878E-97A748ED2869}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add a note for update frequency
</commit_message>
<xml_diff>
--- a/raw_source_inventory.xlsx
+++ b/raw_source_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://centralina-my.sharepoint.com/personal/jliu_centralina_org/Documents/Desktop/mh_explorer/git_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{FA357D76-74AB-4C8A-858B-68E9C7BEB4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91B93D2C-8A80-4002-A4D0-23E702BB2449}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{FA357D76-74AB-4C8A-858B-68E9C7BEB4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3942E6D6-CE27-42BE-B39E-BE07D538CAE3}"/>
   <bookViews>
-    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27675" yWindow="1125" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Sources" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="369">
   <si>
     <t>Raw Data Source Inventory</t>
   </si>
@@ -1124,6 +1124,9 @@
   </si>
   <si>
     <t>CATS, 2026 August</t>
+  </si>
+  <si>
+    <t>monthly check, as needed</t>
   </si>
 </sst>
 </file>
@@ -1204,11 +1207,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1234,13 +1237,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RawSourcesTable" displayName="RawSourcesTable" ref="A3:O60">
-  <autoFilter ref="A3:O60" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
-    <filterColumn colId="10">
-      <filters>
-        <filter val="monthly"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A3:O60" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Source Group"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Raw Item ID"/>
@@ -1422,26 +1419,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="12.4" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
     </row>
     <row r="3" spans="1:18" ht="14.25" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -1490,7 +1487,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="4" spans="1:18" ht="32.1" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -1533,7 +1530,7 @@
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="5" spans="1:18" ht="32.1" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -1576,7 +1573,7 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="6" spans="1:18" ht="32.1" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
@@ -1619,7 +1616,7 @@
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="7" spans="1:18" ht="32.1" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
@@ -1662,7 +1659,7 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="8" spans="1:18" ht="32.1" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
@@ -1705,7 +1702,7 @@
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="9" spans="1:18" ht="32.1" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>42</v>
       </c>
@@ -1752,7 +1749,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="10" spans="1:18" ht="32.1" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>42</v>
       </c>
@@ -1799,7 +1796,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="11" spans="1:18" ht="32.1" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>60</v>
       </c>
@@ -1844,7 +1841,7 @@
       </c>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="12" spans="1:18" ht="32.1" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
@@ -1889,7 +1886,7 @@
       </c>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="13" spans="1:18" ht="32.1" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -1934,7 +1931,7 @@
       </c>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="14" spans="1:18" ht="32.1" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>60</v>
       </c>
@@ -1979,7 +1976,7 @@
       </c>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="15" spans="1:18" ht="32.1" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>60</v>
       </c>
@@ -2024,7 +2021,7 @@
       </c>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:18" ht="32.1" hidden="1" customHeight="1">
+    <row r="16" spans="1:18" ht="32.1" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>60</v>
       </c>
@@ -2069,7 +2066,7 @@
       </c>
       <c r="O16" s="2"/>
     </row>
-    <row r="17" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="17" spans="1:15" ht="32.1" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -2114,7 +2111,7 @@
       </c>
       <c r="O17" s="2"/>
     </row>
-    <row r="18" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="18" spans="1:15" ht="32.1" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>60</v>
       </c>
@@ -2159,7 +2156,7 @@
       </c>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="19" spans="1:15" ht="32.1" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
@@ -2204,7 +2201,7 @@
       </c>
       <c r="O19" s="2"/>
     </row>
-    <row r="20" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="20" spans="1:15" ht="32.1" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>60</v>
       </c>
@@ -2251,7 +2248,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="21" spans="1:15" ht="32.1" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>107</v>
       </c>
@@ -2298,7 +2295,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="22" spans="1:15" ht="32.1" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -2345,7 +2342,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="23" spans="1:15" ht="32.1" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>115</v>
       </c>
@@ -2390,7 +2387,7 @@
       </c>
       <c r="O23" s="2"/>
     </row>
-    <row r="24" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="24" spans="1:15" ht="32.1" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>115</v>
       </c>
@@ -2435,7 +2432,7 @@
       </c>
       <c r="O24" s="2"/>
     </row>
-    <row r="25" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="25" spans="1:15" ht="32.1" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>115</v>
       </c>
@@ -2480,7 +2477,7 @@
       </c>
       <c r="O25" s="2"/>
     </row>
-    <row r="26" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="26" spans="1:15" ht="32.1" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>115</v>
       </c>
@@ -2525,7 +2522,7 @@
       </c>
       <c r="O26" s="2"/>
     </row>
-    <row r="27" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="27" spans="1:15" ht="32.1" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>115</v>
       </c>
@@ -2570,7 +2567,7 @@
       </c>
       <c r="O27" s="2"/>
     </row>
-    <row r="28" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="28" spans="1:15" ht="32.1" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>115</v>
       </c>
@@ -2615,7 +2612,7 @@
       </c>
       <c r="O28" s="2"/>
     </row>
-    <row r="29" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="29" spans="1:15" ht="32.1" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>115</v>
       </c>
@@ -2660,7 +2657,7 @@
       </c>
       <c r="O29" s="2"/>
     </row>
-    <row r="30" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="30" spans="1:15" ht="32.1" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>115</v>
       </c>
@@ -2705,7 +2702,7 @@
       </c>
       <c r="O30" s="2"/>
     </row>
-    <row r="31" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="31" spans="1:15" ht="32.1" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>159</v>
       </c>
@@ -2750,7 +2747,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="32" spans="1:15" ht="32.1" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>163</v>
       </c>
@@ -2832,7 +2829,7 @@
       <c r="L33" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="M33" s="6" t="s">
+      <c r="M33" s="5" t="s">
         <v>174</v>
       </c>
       <c r="N33" s="2" t="s">
@@ -2885,7 +2882,7 @@
       </c>
       <c r="O34" s="2"/>
     </row>
-    <row r="35" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="35" spans="1:15" ht="32.1" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>168</v>
       </c>
@@ -2930,7 +2927,7 @@
       </c>
       <c r="O35" s="2"/>
     </row>
-    <row r="36" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="36" spans="1:15" ht="32.1" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>168</v>
       </c>
@@ -2975,7 +2972,7 @@
       </c>
       <c r="O36" s="2"/>
     </row>
-    <row r="37" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="37" spans="1:15" ht="32.1" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>168</v>
       </c>
@@ -3020,7 +3017,7 @@
       </c>
       <c r="O37" s="2"/>
     </row>
-    <row r="38" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="38" spans="1:15" ht="32.1" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>168</v>
       </c>
@@ -3065,7 +3062,7 @@
       </c>
       <c r="O38" s="2"/>
     </row>
-    <row r="39" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="39" spans="1:15" ht="32.1" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>168</v>
       </c>
@@ -3110,7 +3107,7 @@
       </c>
       <c r="O39" s="2"/>
     </row>
-    <row r="40" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="40" spans="1:15" ht="32.1" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>168</v>
       </c>
@@ -3155,7 +3152,7 @@
       </c>
       <c r="O40" s="2"/>
     </row>
-    <row r="41" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="41" spans="1:15" ht="32.1" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>168</v>
       </c>
@@ -3200,7 +3197,7 @@
       </c>
       <c r="O41" s="2"/>
     </row>
-    <row r="42" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="42" spans="1:15" ht="32.1" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>168</v>
       </c>
@@ -3245,7 +3242,7 @@
       </c>
       <c r="O42" s="2"/>
     </row>
-    <row r="43" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="43" spans="1:15" ht="32.1" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>168</v>
       </c>
@@ -3290,7 +3287,7 @@
       </c>
       <c r="O43" s="2"/>
     </row>
-    <row r="44" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="44" spans="1:15" ht="32.1" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>168</v>
       </c>
@@ -3335,7 +3332,7 @@
       </c>
       <c r="O44" s="2"/>
     </row>
-    <row r="45" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="45" spans="1:15" ht="32.1" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>168</v>
       </c>
@@ -3380,7 +3377,7 @@
       </c>
       <c r="O45" s="2"/>
     </row>
-    <row r="46" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="46" spans="1:15" ht="32.1" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>168</v>
       </c>
@@ -3425,7 +3422,7 @@
       </c>
       <c r="O46" s="2"/>
     </row>
-    <row r="47" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="47" spans="1:15" ht="32.1" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>168</v>
       </c>
@@ -3470,7 +3467,7 @@
       </c>
       <c r="O47" s="2"/>
     </row>
-    <row r="48" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="48" spans="1:15" ht="32.1" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>168</v>
       </c>
@@ -3515,7 +3512,7 @@
       </c>
       <c r="O48" s="2"/>
     </row>
-    <row r="49" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="49" spans="1:15" ht="32.1" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>168</v>
       </c>
@@ -3560,7 +3557,7 @@
       </c>
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="50" spans="1:15" ht="32.1" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>168</v>
       </c>
@@ -3605,7 +3602,7 @@
       </c>
       <c r="O50" s="2"/>
     </row>
-    <row r="51" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="51" spans="1:15" ht="32.1" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>168</v>
       </c>
@@ -3650,7 +3647,7 @@
       </c>
       <c r="O51" s="2"/>
     </row>
-    <row r="52" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="52" spans="1:15" ht="32.1" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>168</v>
       </c>
@@ -3695,7 +3692,7 @@
       </c>
       <c r="O52" s="2"/>
     </row>
-    <row r="53" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="53" spans="1:15" ht="32.1" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>168</v>
       </c>
@@ -3738,7 +3735,7 @@
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="54" spans="1:15" ht="32.1" customHeight="1">
       <c r="A54" s="2" t="s">
         <v>168</v>
       </c>
@@ -3781,7 +3778,7 @@
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="55" spans="1:15" ht="32.1" customHeight="1">
       <c r="A55" s="2" t="s">
         <v>168</v>
       </c>
@@ -3856,12 +3853,12 @@
         <v>283</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>173</v>
+        <v>368</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="M56" s="6" t="s">
+      <c r="M56" s="5" t="s">
         <v>284</v>
       </c>
       <c r="N56" s="2" t="s">
@@ -3869,7 +3866,7 @@
       </c>
       <c r="O56" s="2"/>
     </row>
-    <row r="57" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="57" spans="1:15" ht="32.1" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>279</v>
       </c>
@@ -3912,7 +3909,7 @@
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="58" spans="1:15" ht="32.1" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>279</v>
       </c>
@@ -3955,7 +3952,7 @@
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="1:15" ht="32.1" hidden="1" customHeight="1">
+    <row r="59" spans="1:15" ht="32.1" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>279</v>
       </c>
@@ -4030,7 +4027,7 @@
         <v>304</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>173</v>
+        <v>368</v>
       </c>
       <c r="L60" s="2" t="s">
         <v>26</v>
@@ -4038,7 +4035,7 @@
       <c r="M60" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="N60" s="6" t="s">
+      <c r="N60" s="5" t="s">
         <v>306</v>
       </c>
       <c r="O60" s="2"/>

</xml_diff>